<commit_message>
fix fsh error bae3ebabad1b7f3ef14e191ebbe295ad9afb4ab6
</commit_message>
<xml_diff>
--- a/ig/nr-fix-typo-practioner/StructureDefinition-fr-core-role-code-categorie-professionnelle.xlsx
+++ b/ig/nr-fix-typo-practioner/StructureDefinition-fr-core-role-code-categorie-professionnelle.xlsx
@@ -36,13 +36,13 @@
     <t>Name</t>
   </si>
   <si>
-    <t>FrCorePractitionerRoleCodeCategorieProfessionnelle</t>
+    <t>FRCorePractitionerRoleCodeCategorieProfessionnelle</t>
   </si>
   <si>
     <t>Title</t>
   </si>
   <si>
-    <t>Fr Core Practitioner Role Code Categorie Professionnelle</t>
+    <t>FR Core Practitioner Role Code Categorie Professionnelle</t>
   </si>
   <si>
     <t>Status</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-06T12:47:09+00:00</t>
+    <t>2024-03-06T12:57:57+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>